<commit_message>
added new Test case for contact details
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>Title</t>
   </si>
@@ -78,7 +78,25 @@
     <t>Delete</t>
   </si>
   <si>
-    <t>yuyuuy</t>
+    <t>Contact</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>LastName</t>
+  </si>
+  <si>
+    <t>MiddleName</t>
+  </si>
+  <si>
+    <t>Test Omkar</t>
+  </si>
+  <si>
+    <t>Khopade</t>
+  </si>
+  <si>
+    <t>Maruti</t>
   </si>
 </sst>
 </file>
@@ -404,7 +422,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -415,9 +433,12 @@
     <col min="8" max="8" width="48.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.28515625" customWidth="1"/>
     <col min="10" max="10" width="13.85546875" customWidth="1"/>
+    <col min="11" max="11" width="11" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -449,10 +470,16 @@
         <v>7</v>
       </c>
       <c r="K1" t="s">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="L1" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -482,6 +509,23 @@
       </c>
       <c r="J2" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="b">
+        <v>1</v>
+      </c>
+      <c r="K3" t="s">
+        <v>23</v>
+      </c>
+      <c r="L3" t="s">
+        <v>24</v>
+      </c>
+      <c r="M3" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>